<commit_message>
pref differences excluded, BPP with pp now
</commit_message>
<xml_diff>
--- a/data/MODFLOW_layers_priors.xlsx
+++ b/data/MODFLOW_layers_priors.xlsx
@@ -1,23 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lima0055\Documents\MLAC-3D-HT\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAF4FC9A-6478-4515-BC03-C3710921FE30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="3 layers model"/>
+    <sheet name="3 layers model" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'3 layers model'!$D$1:$D$1000</definedName>
   </definedNames>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="49">
   <si>
     <t>borehole</t>
   </si>
@@ -119,14 +125,58 @@
   </si>
   <si>
     <t>average between (1.51673, 0.11113, 0.10162, 0.10596)</t>
+  </si>
+  <si>
+    <t>OW24P</t>
+  </si>
+  <si>
+    <t>Slug test 2025</t>
+  </si>
+  <si>
+    <t>PMW-2</t>
+  </si>
+  <si>
+    <t>OW17P</t>
+  </si>
+  <si>
+    <t>MW5</t>
+  </si>
+  <si>
+    <t>OW23P</t>
+  </si>
+  <si>
+    <t>OW25P</t>
+  </si>
+  <si>
+    <t>PMW-10</t>
+  </si>
+  <si>
+    <t>PMW-9</t>
+  </si>
+  <si>
+    <t>OW16P</t>
+  </si>
+  <si>
+    <t>OW22P</t>
+  </si>
+  <si>
+    <t>PMW-3</t>
+  </si>
+  <si>
+    <t>PMW-4</t>
+  </si>
+  <si>
+    <t>PMW-5</t>
+  </si>
+  <si>
+    <t>PMW-6</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -140,6 +190,18 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -150,7 +212,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFffe599"/>
+        <fgColor rgb="FFFFE599"/>
       </patternFill>
     </fill>
   </fills>
@@ -171,16 +233,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </left>
       <right style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </right>
       <top style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -188,53 +250,59 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+  <cellXfs count="14">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -245,10 +313,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
@@ -286,71 +354,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -378,7 +446,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -401,11 +469,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -414,13 +482,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -430,7 +498,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -439,7 +507,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -448,7 +516,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -456,10 +524,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -524,23 +592,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="10" width="19.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="13.5703125" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -563,7 +629,7 @@
         <v>6</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -577,14 +643,13 @@
         <v>1</v>
       </c>
       <c r="E2" s="5">
-        <v>0.15638</v>
+        <v>0.15637999999999999</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    </row>
+    <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -598,14 +663,13 @@
         <v>2</v>
       </c>
       <c r="E3" s="5">
-        <v>9.1584</v>
+        <v>9.1584000000000003</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    </row>
+    <row r="4" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -619,14 +683,13 @@
         <v>3</v>
       </c>
       <c r="E4" s="5">
-        <v>0.04208</v>
+        <v>4.2079999999999999E-2</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    </row>
+    <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -640,7 +703,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="5">
-        <v>17.6256</v>
+        <v>17.625599999999999</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>8</v>
@@ -649,7 +712,7 @@
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row r="6" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
@@ -668,9 +731,8 @@
       <c r="F6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    </row>
+    <row r="7" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
@@ -683,7 +745,7 @@
       <c r="D7" s="4">
         <v>3</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="1" t="s">
@@ -693,7 +755,7 @@
         <v>12</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row r="8" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
@@ -706,17 +768,17 @@
       <c r="D8" s="4">
         <v>1</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="7">
         <v>12.096</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row r="9" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>13</v>
       </c>
@@ -729,15 +791,14 @@
       <c r="D9" s="4">
         <v>2</v>
       </c>
-      <c r="E9" s="8">
-        <v>5.62464</v>
+      <c r="E9" s="7">
+        <v>5.6246400000000003</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G9" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    </row>
+    <row r="10" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>13</v>
       </c>
@@ -750,7 +811,7 @@
       <c r="D10" s="4">
         <v>3</v>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="7">
         <v>25.862399999999997</v>
       </c>
       <c r="F10" s="1" t="s">
@@ -760,7 +821,7 @@
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row r="11" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
@@ -773,7 +834,7 @@
       <c r="D11" s="4">
         <v>1</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="1" t="s">
@@ -783,7 +844,7 @@
         <v>12</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+    <row r="12" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>16</v>
       </c>
@@ -806,7 +867,7 @@
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row r="13" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>16</v>
       </c>
@@ -820,7 +881,7 @@
         <v>3</v>
       </c>
       <c r="E13" s="5">
-        <v>0.2098625</v>
+        <v>0.20986250000000001</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>17</v>
@@ -829,7 +890,7 @@
         <v>19</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row r="14" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -842,7 +903,7 @@
       <c r="D14" s="4">
         <v>1</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F14" s="1" t="s">
@@ -852,7 +913,7 @@
         <v>12</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+    <row r="15" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>20</v>
       </c>
@@ -866,7 +927,7 @@
         <v>2</v>
       </c>
       <c r="E15" s="5">
-        <v>26.4082725</v>
+        <v>26.408272499999999</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>17</v>
@@ -875,7 +936,7 @@
         <v>21</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+    <row r="16" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>20</v>
       </c>
@@ -898,7 +959,7 @@
         <v>22</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+    <row r="17" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
@@ -911,7 +972,7 @@
       <c r="D17" s="4">
         <v>1</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F17" s="1" t="s">
@@ -921,7 +982,7 @@
         <v>12</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+    <row r="18" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>23</v>
       </c>
@@ -944,7 +1005,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+    <row r="19" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>23</v>
       </c>
@@ -958,7 +1019,7 @@
         <v>3</v>
       </c>
       <c r="E19" s="5">
-        <v>0.2889</v>
+        <v>0.28889999999999999</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>17</v>
@@ -967,7 +1028,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+    <row r="20" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>26</v>
       </c>
@@ -980,7 +1041,7 @@
       <c r="D20" s="4">
         <v>1</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F20" s="1" t="s">
@@ -990,7 +1051,7 @@
         <v>12</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+    <row r="21" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>26</v>
       </c>
@@ -1004,14 +1065,13 @@
         <v>2</v>
       </c>
       <c r="E21" s="5">
-        <v>23.32691</v>
+        <v>23.326910000000002</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G21" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+    </row>
+    <row r="22" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>26</v>
       </c>
@@ -1034,7 +1094,7 @@
         <v>27</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+    <row r="23" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>28</v>
       </c>
@@ -1048,14 +1108,13 @@
         <v>1</v>
       </c>
       <c r="E23" s="5">
-        <v>0.34311</v>
+        <v>0.34311000000000003</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G23" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+    </row>
+    <row r="24" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>28</v>
       </c>
@@ -1069,14 +1128,13 @@
         <v>2</v>
       </c>
       <c r="E24" s="5">
-        <v>51.19549</v>
+        <v>51.195489999999999</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G24" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+    </row>
+    <row r="25" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>28</v>
       </c>
@@ -1099,7 +1157,7 @@
         <v>29</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+    <row r="26" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>30</v>
       </c>
@@ -1113,14 +1171,13 @@
         <v>1</v>
       </c>
       <c r="E26" s="5">
-        <v>16.6827</v>
+        <v>16.682700000000001</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G26" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
+    </row>
+    <row r="27" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>30</v>
       </c>
@@ -1134,14 +1191,13 @@
         <v>2</v>
       </c>
       <c r="E27" s="5">
-        <v>16.89796</v>
+        <v>16.897960000000001</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G27" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
+    </row>
+    <row r="28" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>30</v>
       </c>
@@ -1164,7 +1220,7 @@
         <v>31</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
+    <row r="29" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>32</v>
       </c>
@@ -1183,9 +1239,8 @@
       <c r="F29" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G29" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
+    </row>
+    <row r="30" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>32</v>
       </c>
@@ -1204,9 +1259,8 @@
       <c r="F30" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G30" s="6"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
+    </row>
+    <row r="31" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>32</v>
       </c>
@@ -1220,7 +1274,7 @@
         <v>3</v>
       </c>
       <c r="E31" s="5">
-        <v>0.45886</v>
+        <v>0.45885999999999999</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>17</v>
@@ -1229,7 +1283,289 @@
         <v>33</v>
       </c>
     </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="12">
+        <v>4980200</v>
+      </c>
+      <c r="C32" s="12">
+        <v>480646</v>
+      </c>
+      <c r="D32" s="12">
+        <v>2</v>
+      </c>
+      <c r="E32" s="13">
+        <v>8.49</v>
+      </c>
+      <c r="F32" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B33" s="12">
+        <v>4980249</v>
+      </c>
+      <c r="C33" s="12">
+        <v>480650</v>
+      </c>
+      <c r="D33" s="12">
+        <v>2</v>
+      </c>
+      <c r="E33" s="13">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="F33" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B34" s="12">
+        <v>4980246</v>
+      </c>
+      <c r="C34" s="12">
+        <v>480722</v>
+      </c>
+      <c r="D34" s="12">
+        <v>2</v>
+      </c>
+      <c r="E34" s="13">
+        <v>10.43</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B35" s="12">
+        <v>4980166</v>
+      </c>
+      <c r="C35" s="12">
+        <v>480647</v>
+      </c>
+      <c r="D35" s="12">
+        <v>2</v>
+      </c>
+      <c r="E35" s="13">
+        <v>6.5000000000000002E-2</v>
+      </c>
+      <c r="F35" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B36" s="12">
+        <v>4980077</v>
+      </c>
+      <c r="C36" s="12">
+        <v>480655</v>
+      </c>
+      <c r="D36" s="12">
+        <v>2</v>
+      </c>
+      <c r="E36" s="13">
+        <v>1.44</v>
+      </c>
+      <c r="F36" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B37" s="12">
+        <v>4980202</v>
+      </c>
+      <c r="C37" s="12">
+        <v>480810</v>
+      </c>
+      <c r="D37" s="12">
+        <v>2</v>
+      </c>
+      <c r="E37" s="13">
+        <v>0.25</v>
+      </c>
+      <c r="F37" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B38" s="12">
+        <v>4980041</v>
+      </c>
+      <c r="C38" s="12">
+        <v>480775</v>
+      </c>
+      <c r="D38" s="12">
+        <v>2</v>
+      </c>
+      <c r="E38" s="13">
+        <v>3.9E-2</v>
+      </c>
+      <c r="F38" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" s="12">
+        <v>4980125</v>
+      </c>
+      <c r="C39" s="12">
+        <v>480867</v>
+      </c>
+      <c r="D39" s="12">
+        <v>2</v>
+      </c>
+      <c r="E39" s="13">
+        <v>0.13800000000000001</v>
+      </c>
+      <c r="F39" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B40" s="12">
+        <v>4980166</v>
+      </c>
+      <c r="C40" s="12">
+        <v>480814</v>
+      </c>
+      <c r="D40" s="12">
+        <v>2</v>
+      </c>
+      <c r="E40" s="13">
+        <v>0.54100000000000004</v>
+      </c>
+      <c r="F40" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B41" s="12">
+        <v>4980130</v>
+      </c>
+      <c r="C41" s="12">
+        <v>480720</v>
+      </c>
+      <c r="D41" s="12">
+        <v>2</v>
+      </c>
+      <c r="E41" s="13">
+        <v>138.5</v>
+      </c>
+      <c r="F41" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B42" s="12">
+        <v>4980128</v>
+      </c>
+      <c r="C42" s="12">
+        <v>480773</v>
+      </c>
+      <c r="D42" s="12">
+        <v>2</v>
+      </c>
+      <c r="E42" s="13">
+        <v>67.709999999999994</v>
+      </c>
+      <c r="F42" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B43" s="12">
+        <v>4979962</v>
+      </c>
+      <c r="C43" s="12">
+        <v>480878</v>
+      </c>
+      <c r="D43" s="12">
+        <v>2</v>
+      </c>
+      <c r="E43" s="13">
+        <v>2.27</v>
+      </c>
+      <c r="F43" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B44" s="12">
+        <v>4979939</v>
+      </c>
+      <c r="C44" s="12">
+        <v>480768</v>
+      </c>
+      <c r="D44" s="12">
+        <v>2</v>
+      </c>
+      <c r="E44" s="13">
+        <v>39.880000000000003</v>
+      </c>
+      <c r="F44" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B45" s="12">
+        <v>4980073</v>
+      </c>
+      <c r="C45" s="12">
+        <v>480717</v>
+      </c>
+      <c r="D45" s="12">
+        <v>2</v>
+      </c>
+      <c r="E45" s="13">
+        <v>131.07</v>
+      </c>
+      <c r="F45" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
MODFLOW folder structure created, with in and out files outside, process of including all injection tests
</commit_message>
<xml_diff>
--- a/data/MODFLOW_layers_priors.xlsx
+++ b/data/MODFLOW_layers_priors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lima0055\Documents\MLAC-3D-HT\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAF4FC9A-6478-4515-BC03-C3710921FE30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADDB371D-88ED-4285-B324-8ABDAAC92B3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="3 layers model" sheetId="1" r:id="rId1"/>
@@ -18,12 +18,25 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'3 layers model'!$D$1:$D$1000</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="60">
   <si>
     <t>borehole</t>
   </si>
@@ -170,6 +183,39 @@
   </si>
   <si>
     <t>PMW-6</t>
+  </si>
+  <si>
+    <t>PMW-1</t>
+  </si>
+  <si>
+    <t>method</t>
+  </si>
+  <si>
+    <t>packer test</t>
+  </si>
+  <si>
+    <t>slug test</t>
+  </si>
+  <si>
+    <t>pumping test</t>
+  </si>
+  <si>
+    <t>PEER 1999, average between K estimation for different analytical solution</t>
+  </si>
+  <si>
+    <t>packer + pumping test</t>
+  </si>
+  <si>
+    <t>pumping test (PEER, 1999)</t>
+  </si>
+  <si>
+    <t>PZ-1</t>
+  </si>
+  <si>
+    <t>old value</t>
+  </si>
+  <si>
+    <t>slug + pumping test</t>
   </si>
 </sst>
 </file>
@@ -250,7 +296,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -282,15 +328,19 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -596,17 +646,19 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I47"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="13.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" style="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="13.5546875" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5546875" style="10" customWidth="1"/>
+    <col min="7" max="7" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.88671875" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -622,14 +674,20 @@
       <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I1" s="15" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -645,11 +703,14 @@
       <c r="E2" s="5">
         <v>0.15637999999999999</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -663,13 +724,16 @@
         <v>2</v>
       </c>
       <c r="E3" s="5">
-        <v>9.1584000000000003</v>
-      </c>
-      <c r="F3" s="1" t="s">
+        <v>8.5</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -685,11 +749,14 @@
       <c r="E4" s="5">
         <v>4.2079999999999999E-2</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -705,14 +772,17 @@
       <c r="E5" s="5">
         <v>17.625599999999999</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
@@ -728,11 +798,14 @@
       <c r="E6" s="5">
         <v>24.9696</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
@@ -748,14 +821,17 @@
       <c r="E7" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
@@ -768,17 +844,20 @@
       <c r="D8" s="4">
         <v>1</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="14">
         <v>12.096</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="H8" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>13</v>
       </c>
@@ -791,14 +870,17 @@
       <c r="D9" s="4">
         <v>2</v>
       </c>
-      <c r="E9" s="7">
-        <v>5.6246400000000003</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E9" s="14">
+        <v>19.100000000000001</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>13</v>
       </c>
@@ -814,14 +896,17 @@
       <c r="E10" s="7">
         <v>25.862399999999997</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
@@ -837,14 +922,17 @@
       <c r="E11" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>17</v>
+      <c r="F11" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="G11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>16</v>
       </c>
@@ -860,14 +948,17 @@
       <c r="E12" s="5">
         <v>7.0922149999999995</v>
       </c>
-      <c r="F12" s="1" t="s">
-        <v>17</v>
+      <c r="F12" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="G12" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H12" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>16</v>
       </c>
@@ -883,14 +974,17 @@
       <c r="E13" s="5">
         <v>0.20986250000000001</v>
       </c>
-      <c r="F13" s="1" t="s">
-        <v>17</v>
+      <c r="F13" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="G13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H13" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -906,14 +1000,17 @@
       <c r="E14" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F14" s="1" t="s">
-        <v>17</v>
+      <c r="F14" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="G14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>20</v>
       </c>
@@ -929,14 +1026,17 @@
       <c r="E15" s="5">
         <v>26.408272499999999</v>
       </c>
-      <c r="F15" s="1" t="s">
-        <v>17</v>
+      <c r="F15" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="G15" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H15" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>20</v>
       </c>
@@ -952,14 +1052,17 @@
       <c r="E16" s="5">
         <v>0.23786666666666667</v>
       </c>
-      <c r="F16" s="1" t="s">
-        <v>17</v>
+      <c r="F16" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="G16" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H16" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
@@ -975,14 +1078,17 @@
       <c r="E17" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>17</v>
+      <c r="F17" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="G17" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>23</v>
       </c>
@@ -998,14 +1104,17 @@
       <c r="E18" s="5">
         <v>30.443694999999998</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>17</v>
+      <c r="F18" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="G18" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>23</v>
       </c>
@@ -1021,14 +1130,17 @@
       <c r="E19" s="5">
         <v>0.28889999999999999</v>
       </c>
-      <c r="F19" s="1" t="s">
-        <v>17</v>
+      <c r="F19" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="G19" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H19" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>26</v>
       </c>
@@ -1044,14 +1156,17 @@
       <c r="E20" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F20" s="1" t="s">
-        <v>17</v>
+      <c r="F20" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="G20" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H20" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>26</v>
       </c>
@@ -1067,11 +1182,14 @@
       <c r="E21" s="5">
         <v>23.326910000000002</v>
       </c>
-      <c r="F21" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F21" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>26</v>
       </c>
@@ -1087,14 +1205,17 @@
       <c r="E22" s="5">
         <v>3.2745150000000005</v>
       </c>
-      <c r="F22" s="1" t="s">
-        <v>17</v>
+      <c r="F22" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="G22" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H22" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>28</v>
       </c>
@@ -1110,11 +1231,14 @@
       <c r="E23" s="5">
         <v>0.34311000000000003</v>
       </c>
-      <c r="F23" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F23" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>28</v>
       </c>
@@ -1130,11 +1254,14 @@
       <c r="E24" s="5">
         <v>51.195489999999999</v>
       </c>
-      <c r="F24" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F24" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>28</v>
       </c>
@@ -1150,14 +1277,17 @@
       <c r="E25" s="5">
         <v>0.14970333333333333</v>
       </c>
-      <c r="F25" s="1" t="s">
-        <v>17</v>
+      <c r="F25" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="G25" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H25" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>30</v>
       </c>
@@ -1173,11 +1303,14 @@
       <c r="E26" s="5">
         <v>16.682700000000001</v>
       </c>
-      <c r="F26" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F26" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>30</v>
       </c>
@@ -1193,11 +1326,14 @@
       <c r="E27" s="5">
         <v>16.897960000000001</v>
       </c>
-      <c r="F27" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F27" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>30</v>
       </c>
@@ -1213,14 +1349,17 @@
       <c r="E28" s="5">
         <v>0.8798433333333332</v>
       </c>
-      <c r="F28" s="1" t="s">
-        <v>17</v>
+      <c r="F28" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="G28" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H28" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>32</v>
       </c>
@@ -1236,11 +1375,14 @@
       <c r="E29" s="5">
         <v>18.18656</v>
       </c>
-      <c r="F29" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F29" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>32</v>
       </c>
@@ -1256,11 +1398,14 @@
       <c r="E30" s="5">
         <v>12.19326</v>
       </c>
-      <c r="F30" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F30" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>32</v>
       </c>
@@ -1276,291 +1421,397 @@
       <c r="E31" s="5">
         <v>0.45885999999999999</v>
       </c>
-      <c r="F31" s="1" t="s">
-        <v>17</v>
+      <c r="F31" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="G31" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H31" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="11" t="s">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A32" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B32" s="12">
+      <c r="B32" s="11">
         <v>4980200</v>
       </c>
-      <c r="C32" s="12">
+      <c r="C32" s="11">
         <v>480646</v>
       </c>
-      <c r="D32" s="12">
-        <v>2</v>
-      </c>
-      <c r="E32" s="13">
+      <c r="D32" s="11">
+        <v>2</v>
+      </c>
+      <c r="E32" s="12">
         <v>8.49</v>
       </c>
-      <c r="F32" s="11" t="s">
+      <c r="F32" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G32" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="11" t="s">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B33" s="12">
+      <c r="B33" s="11">
         <v>4980249</v>
       </c>
-      <c r="C33" s="12">
+      <c r="C33" s="11">
         <v>480650</v>
       </c>
-      <c r="D33" s="12">
-        <v>2</v>
-      </c>
-      <c r="E33" s="13">
+      <c r="D33" s="11">
+        <v>2</v>
+      </c>
+      <c r="E33" s="12">
+        <v>16.07</v>
+      </c>
+      <c r="F33" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I33" s="15">
         <v>1.1100000000000001</v>
       </c>
-      <c r="F33" s="11" t="s">
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B34" s="11">
+        <v>4980246</v>
+      </c>
+      <c r="C34" s="11">
+        <v>480722</v>
+      </c>
+      <c r="D34" s="11">
+        <v>2</v>
+      </c>
+      <c r="E34" s="12">
+        <v>10.43</v>
+      </c>
+      <c r="F34" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G34" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="B34" s="12">
-        <v>4980246</v>
-      </c>
-      <c r="C34" s="12">
-        <v>480722</v>
-      </c>
-      <c r="D34" s="12">
-        <v>2</v>
-      </c>
-      <c r="E34" s="13">
-        <v>10.43</v>
-      </c>
-      <c r="F34" s="11" t="s">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B35" s="11">
+        <v>4980166</v>
+      </c>
+      <c r="C35" s="11">
+        <v>480647</v>
+      </c>
+      <c r="D35" s="11">
+        <v>2</v>
+      </c>
+      <c r="E35" s="12">
+        <v>6.5000000000000002E-2</v>
+      </c>
+      <c r="F35" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G35" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B35" s="12">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A36" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B36" s="11">
+        <v>4980077</v>
+      </c>
+      <c r="C36" s="11">
+        <v>480655</v>
+      </c>
+      <c r="D36" s="11">
+        <v>2</v>
+      </c>
+      <c r="E36" s="12">
+        <v>1.44</v>
+      </c>
+      <c r="F36" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B37" s="11">
+        <v>4980202</v>
+      </c>
+      <c r="C37" s="11">
+        <v>480810</v>
+      </c>
+      <c r="D37" s="11">
+        <v>2</v>
+      </c>
+      <c r="E37" s="12">
+        <v>0.25</v>
+      </c>
+      <c r="F37" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A38" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B38" s="11">
+        <v>4980041</v>
+      </c>
+      <c r="C38" s="11">
+        <v>480775</v>
+      </c>
+      <c r="D38" s="11">
+        <v>2</v>
+      </c>
+      <c r="E38" s="12">
+        <v>3.9E-2</v>
+      </c>
+      <c r="F38" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A39" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" s="11">
+        <v>4980125</v>
+      </c>
+      <c r="C39" s="11">
+        <v>480867</v>
+      </c>
+      <c r="D39" s="11">
+        <v>2</v>
+      </c>
+      <c r="E39" s="12">
+        <v>0.13800000000000001</v>
+      </c>
+      <c r="F39" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A40" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B40" s="11">
         <v>4980166</v>
       </c>
-      <c r="C35" s="12">
-        <v>480647</v>
-      </c>
-      <c r="D35" s="12">
-        <v>2</v>
-      </c>
-      <c r="E35" s="13">
-        <v>6.5000000000000002E-2</v>
-      </c>
-      <c r="F35" s="11" t="s">
+      <c r="C40" s="11">
+        <v>480814</v>
+      </c>
+      <c r="D40" s="11">
+        <v>2</v>
+      </c>
+      <c r="E40" s="12">
+        <v>0.54100000000000004</v>
+      </c>
+      <c r="F40" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G40" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B36" s="12">
-        <v>4980077</v>
-      </c>
-      <c r="C36" s="12">
-        <v>480655</v>
-      </c>
-      <c r="D36" s="12">
-        <v>2</v>
-      </c>
-      <c r="E36" s="13">
-        <v>1.44</v>
-      </c>
-      <c r="F36" s="11" t="s">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B41" s="11">
+        <v>4980130</v>
+      </c>
+      <c r="C41" s="11">
+        <v>480720</v>
+      </c>
+      <c r="D41" s="11">
+        <v>2</v>
+      </c>
+      <c r="E41" s="12">
+        <v>138.5</v>
+      </c>
+      <c r="F41" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G41" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="B37" s="12">
-        <v>4980202</v>
-      </c>
-      <c r="C37" s="12">
-        <v>480810</v>
-      </c>
-      <c r="D37" s="12">
-        <v>2</v>
-      </c>
-      <c r="E37" s="13">
-        <v>0.25</v>
-      </c>
-      <c r="F37" s="11" t="s">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B42" s="11">
+        <v>4980128</v>
+      </c>
+      <c r="C42" s="11">
+        <v>480773</v>
+      </c>
+      <c r="D42" s="11">
+        <v>2</v>
+      </c>
+      <c r="E42" s="12">
+        <v>32.83</v>
+      </c>
+      <c r="F42" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G42" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B38" s="12">
-        <v>4980041</v>
-      </c>
-      <c r="C38" s="12">
-        <v>480775</v>
-      </c>
-      <c r="D38" s="12">
-        <v>2</v>
-      </c>
-      <c r="E38" s="13">
-        <v>3.9E-2</v>
-      </c>
-      <c r="F38" s="11" t="s">
+      <c r="I42" s="12">
+        <v>67.709999999999994</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A43" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B43" s="11">
+        <v>4979962</v>
+      </c>
+      <c r="C43" s="11">
+        <v>480878</v>
+      </c>
+      <c r="D43" s="11">
+        <v>2</v>
+      </c>
+      <c r="E43" s="12">
+        <v>27.9</v>
+      </c>
+      <c r="F43" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G43" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="B39" s="12">
-        <v>4980125</v>
-      </c>
-      <c r="C39" s="12">
-        <v>480867</v>
-      </c>
-      <c r="D39" s="12">
-        <v>2</v>
-      </c>
-      <c r="E39" s="13">
-        <v>0.13800000000000001</v>
-      </c>
-      <c r="F39" s="11" t="s">
+      <c r="I43" s="12">
+        <v>2.27</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A44" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B44" s="11">
+        <v>4979939</v>
+      </c>
+      <c r="C44" s="11">
+        <v>480768</v>
+      </c>
+      <c r="D44" s="11">
+        <v>2</v>
+      </c>
+      <c r="E44" s="12">
+        <v>39.479999999999997</v>
+      </c>
+      <c r="F44" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G44" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="B40" s="12">
-        <v>4980166</v>
-      </c>
-      <c r="C40" s="12">
-        <v>480814</v>
-      </c>
-      <c r="D40" s="12">
-        <v>2</v>
-      </c>
-      <c r="E40" s="13">
-        <v>0.54100000000000004</v>
-      </c>
-      <c r="F40" s="11" t="s">
+      <c r="I44" s="12">
+        <v>39.880000000000003</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A45" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B45" s="11">
+        <v>4980073</v>
+      </c>
+      <c r="C45" s="11">
+        <v>480717</v>
+      </c>
+      <c r="D45" s="11">
+        <v>2</v>
+      </c>
+      <c r="E45" s="12">
+        <v>18.309999999999999</v>
+      </c>
+      <c r="F45" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G45" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B41" s="12">
-        <v>4980130</v>
-      </c>
-      <c r="C41" s="12">
-        <v>480720</v>
-      </c>
-      <c r="D41" s="12">
-        <v>2</v>
-      </c>
-      <c r="E41" s="13">
-        <v>138.5</v>
-      </c>
-      <c r="F41" s="11" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="B42" s="12">
-        <v>4980128</v>
-      </c>
-      <c r="C42" s="12">
-        <v>480773</v>
-      </c>
-      <c r="D42" s="12">
-        <v>2</v>
-      </c>
-      <c r="E42" s="13">
-        <v>67.709999999999994</v>
-      </c>
-      <c r="F42" s="11" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="B43" s="12">
-        <v>4979962</v>
-      </c>
-      <c r="C43" s="12">
-        <v>480878</v>
-      </c>
-      <c r="D43" s="12">
-        <v>2</v>
-      </c>
-      <c r="E43" s="13">
-        <v>2.27</v>
-      </c>
-      <c r="F43" s="11" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="B44" s="12">
-        <v>4979939</v>
-      </c>
-      <c r="C44" s="12">
-        <v>480768</v>
-      </c>
-      <c r="D44" s="12">
-        <v>2</v>
-      </c>
-      <c r="E44" s="13">
-        <v>39.880000000000003</v>
-      </c>
-      <c r="F44" s="11" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="B45" s="12">
-        <v>4980073</v>
-      </c>
-      <c r="C45" s="12">
-        <v>480717</v>
-      </c>
-      <c r="D45" s="12">
-        <v>2</v>
-      </c>
-      <c r="E45" s="13">
+      <c r="I45" s="12">
         <v>131.07</v>
       </c>
-      <c r="F45" s="11" t="s">
-        <v>35</v>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A46" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B46" s="11">
+        <v>4980036</v>
+      </c>
+      <c r="C46" s="11">
+        <v>480813</v>
+      </c>
+      <c r="D46" s="11">
+        <v>2</v>
+      </c>
+      <c r="E46" s="12">
+        <v>10.975000000000001</v>
+      </c>
+      <c r="F46" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="G46" s="13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A47" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B47" s="11">
+        <v>4980031</v>
+      </c>
+      <c r="C47" s="11">
+        <v>480820</v>
+      </c>
+      <c r="D47" s="11">
+        <v>2</v>
+      </c>
+      <c r="E47" s="12">
+        <v>32.85</v>
+      </c>
+      <c r="F47" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="G47" s="13" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>